<commit_message>
fix: prioritize Excel 3-tabs reading with READY status, fix Friday theme to living costs, and sync correct dates
</commit_message>
<xml_diff>
--- a/content_ideas_sheet.xlsx
+++ b/content_ideas_sheet.xlsx
@@ -867,7 +867,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
@@ -948,7 +948,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -975,7 +975,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>

</xml_diff>